<commit_message>
Model and exposure spreadsheets for for PFOA were revised to include tabs that match those used in the Bernstein et al. (2021) paper.
</commit_message>
<xml_diff>
--- a/Inputs/PFOA_template_parameters_Model.xlsx
+++ b/Inputs/PFOA_template_parameters_Model.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/bernstein_amanda_epa_gov/Documents/Documents/PKWG_models/pbpk_template_project/Inputs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa.sharepoint.com/sites/ORD/pkwg/Shared Documents/PFAS/PFAS inhalation/pfas_inhalation_pbpk/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="94" documentId="13_ncr:1_{C7746A5F-920D-41F0-A536-A594C5CF14B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8EF6874E-F71F-41D7-9045-3602B84A7742}"/>
+  <xr:revisionPtr revIDLastSave="97" documentId="13_ncr:1_{C7746A5F-920D-41F0-A536-A594C5CF14B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0835F917-0AD2-4EE2-B689-A706E57128C5}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
+    <workbookView xWindow="2265" yWindow="345" windowWidth="21600" windowHeight="11100" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
   </bookViews>
   <sheets>
     <sheet name="MaleRat" sheetId="9" r:id="rId1"/>
@@ -871,10 +871,14 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -912,7 +916,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1018,7 +1022,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1160,7 +1164,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1169,18 +1173,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3ADCAA70-43B6-4F02-AE2A-67A6EACE5958}">
   <dimension ref="A1:F104"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="51" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.08984375" customWidth="1"/>
-    <col min="5" max="5" width="22.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.54296875" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" customWidth="1"/>
+    <col min="5" max="5" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1200,7 +1204,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -1214,7 +1218,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -1225,7 +1229,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
@@ -1236,7 +1240,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -1253,7 +1257,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -1270,7 +1274,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
@@ -1284,7 +1288,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>20</v>
       </c>
@@ -1298,7 +1302,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>236</v>
       </c>
@@ -1315,7 +1319,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>136</v>
       </c>
@@ -1332,7 +1336,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>137</v>
       </c>
@@ -1349,7 +1353,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>180</v>
       </c>
@@ -1366,7 +1370,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>184</v>
       </c>
@@ -1383,7 +1387,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>169</v>
       </c>
@@ -1400,7 +1404,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>198</v>
       </c>
@@ -1418,7 +1422,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>201</v>
       </c>
@@ -1433,7 +1437,7 @@
         <v>0.84000000000000008</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>0</v>
       </c>
@@ -1453,7 +1457,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>71</v>
       </c>
@@ -1470,7 +1474,7 @@
         <v>414.07</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>27</v>
       </c>
@@ -1484,7 +1488,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>29</v>
       </c>
@@ -1498,7 +1502,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>228</v>
       </c>
@@ -1516,7 +1520,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>31</v>
       </c>
@@ -1530,7 +1534,7 @@
         <v>-0.25</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>33</v>
       </c>
@@ -1551,7 +1555,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>43</v>
       </c>
@@ -1562,7 +1566,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>142</v>
       </c>
@@ -1579,7 +1583,7 @@
         <v>270000</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>143</v>
       </c>
@@ -1596,7 +1600,7 @@
         <v>67000</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>48</v>
       </c>
@@ -1614,7 +1618,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>144</v>
       </c>
@@ -1631,7 +1635,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>145</v>
       </c>
@@ -1645,7 +1649,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>146</v>
       </c>
@@ -1662,7 +1666,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>52</v>
       </c>
@@ -1676,7 +1680,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>53</v>
       </c>
@@ -1693,7 +1697,7 @@
         <v>31.3</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>54</v>
       </c>
@@ -1707,7 +1711,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>55</v>
       </c>
@@ -1724,7 +1728,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>170</v>
       </c>
@@ -1738,7 +1742,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>57</v>
       </c>
@@ -1755,7 +1759,7 @@
         <v>634.5</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>225</v>
       </c>
@@ -1769,7 +1773,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>226</v>
       </c>
@@ -1783,7 +1787,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>227</v>
       </c>
@@ -1797,7 +1801,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>147</v>
       </c>
@@ -1811,7 +1815,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>148</v>
       </c>
@@ -1825,7 +1829,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>149</v>
       </c>
@@ -1839,7 +1843,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>150</v>
       </c>
@@ -1853,7 +1857,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>151</v>
       </c>
@@ -1867,7 +1871,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>152</v>
       </c>
@@ -1881,7 +1885,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>153</v>
       </c>
@@ -1895,7 +1899,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>154</v>
       </c>
@@ -1909,7 +1913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>38</v>
       </c>
@@ -1920,7 +1924,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>173</v>
       </c>
@@ -1931,7 +1935,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>40</v>
       </c>
@@ -1942,7 +1946,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>190</v>
       </c>
@@ -1959,7 +1963,7 @@
         <v>7.0499999999999993E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>165</v>
       </c>
@@ -1973,7 +1977,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>166</v>
       </c>
@@ -1984,7 +1988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>204</v>
       </c>
@@ -1998,7 +2002,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>206</v>
       </c>
@@ -2012,7 +2016,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>231</v>
       </c>
@@ -2029,7 +2033,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>42</v>
       </c>
@@ -2043,7 +2047,7 @@
         <v>6.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>0</v>
       </c>
@@ -2060,7 +2064,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>81</v>
       </c>
@@ -2077,7 +2081,7 @@
         <v>3.1199999999999999E-2</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>138</v>
       </c>
@@ -2091,7 +2095,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>140</v>
       </c>
@@ -2105,7 +2109,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>84</v>
       </c>
@@ -2119,7 +2123,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>91</v>
       </c>
@@ -2133,7 +2137,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>92</v>
       </c>
@@ -2150,7 +2154,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>93</v>
       </c>
@@ -2167,7 +2171,7 @@
         <v>8.3999999999999995E-3</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>94</v>
       </c>
@@ -2184,7 +2188,7 @@
         <v>8.4000000000000003E-4</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>95</v>
       </c>
@@ -2198,7 +2202,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>96</v>
       </c>
@@ -2212,7 +2216,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>97</v>
       </c>
@@ -2226,7 +2230,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>98</v>
       </c>
@@ -2240,7 +2244,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>99</v>
       </c>
@@ -2254,7 +2258,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>100</v>
       </c>
@@ -2268,7 +2272,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>155</v>
       </c>
@@ -2286,7 +2290,7 @@
         <v>0.76456000000000002</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>106</v>
       </c>
@@ -2300,7 +2304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>107</v>
       </c>
@@ -2317,7 +2321,7 @@
         <v>0.183</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>108</v>
       </c>
@@ -2334,7 +2338,7 @@
         <v>0.14099999999999999</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>109</v>
       </c>
@@ -2348,7 +2352,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>110</v>
       </c>
@@ -2362,7 +2366,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>111</v>
       </c>
@@ -2376,7 +2380,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>112</v>
       </c>
@@ -2390,7 +2394,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>113</v>
       </c>
@@ -2404,7 +2408,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>114</v>
       </c>
@@ -2418,7 +2422,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>158</v>
       </c>
@@ -2436,7 +2440,7 @@
         <v>0.60549999999999993</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>123</v>
       </c>
@@ -2447,7 +2451,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>124</v>
       </c>
@@ -2458,7 +2462,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>125</v>
       </c>
@@ -2472,7 +2476,7 @@
         <v>2.2000000000000002</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>126</v>
       </c>
@@ -2486,7 +2490,7 @@
         <v>1.05</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>127</v>
       </c>
@@ -2497,7 +2501,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>128</v>
       </c>
@@ -2508,7 +2512,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>129</v>
       </c>
@@ -2519,7 +2523,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>130</v>
       </c>
@@ -2530,7 +2534,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>131</v>
       </c>
@@ -2541,7 +2545,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>132</v>
       </c>
@@ -2552,7 +2556,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>161</v>
       </c>
@@ -2566,7 +2570,7 @@
         <v>0.11</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>0</v>
       </c>
@@ -2583,7 +2587,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>35</v>
       </c>
@@ -2594,7 +2598,7 @@
         <v>0.46</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>0</v>
       </c>
@@ -2609,7 +2613,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
         <v>75</v>
       </c>
@@ -2617,7 +2621,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>77</v>
       </c>
@@ -2625,7 +2629,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
         <v>79</v>
       </c>
@@ -2663,6 +2667,20 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C107526348C97345843FB1F7E3F5FF14" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1f5efa0b4590ceb4068c523eef838cbf">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="2ba80736-48fa-4d73-aaff-bacaeeed013a" xmlns:ns6="41d9f072-86bf-4c63-b117-debf50ff4701" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9d32b47d5805bf9e4ccfb00021215c68" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -3135,7 +3153,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
@@ -3180,25 +3198,46 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76DF7049-5D71-4C8A-9827-79FC4B574086}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76DF7049-5D71-4C8A-9827-79FC4B574086}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
+    <ds:schemaRef ds:uri="41d9f072-86bf-4c63-b117-debf50ff4701"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA939294-F21F-45CD-81A6-3A616888DAC5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -3208,22 +3247,7 @@
     <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
     <ds:schemaRef ds:uri="93237db7-bebb-43bb-9414-bc3313990c09"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>